<commit_message>
결과 파일 업데이트 2026-08-12 10:08
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260812.xlsx
+++ b/results/andar_할인율모니터링_20260812.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7,185</t>
+          <t>7,189</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>265</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>265</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>265</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>212</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>184</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>4,760</t>
+          <t>4,761</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>10,275</t>
+          <t>10,276</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>724</t>
+          <t>728</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>337</t>
+          <t>338</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>226</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>4,760</t>
+          <t>4,761</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>1,519</t>
+          <t>1,520</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -4271,7 +4271,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>473</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>473</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>164</t>
+          <t>165</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>84</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">

</xml_diff>